<commit_message>
analisis funcional login arreglado
</commit_message>
<xml_diff>
--- a/1-Y2K-QA-ANALISIS-FUNCIONAL/DOCUMENTOS/ANALISIS_FUNCIONAL_HU_01_LOGIN_Y2K.xlsx
+++ b/1-Y2K-QA-ANALISIS-FUNCIONAL/DOCUMENTOS/ANALISIS_FUNCIONAL_HU_01_LOGIN_Y2K.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7635" firstSheet="2" activeTab="6"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7635" firstSheet="2" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="HU-01 Historia de Usuario" sheetId="1" r:id="rId1"/>
@@ -2578,29 +2578,29 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2628,10 +2628,10 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2946,502 +2946,502 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="40" t="s">
         <v>683</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="31" t="s">
+      <c r="A4" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="32"/>
-      <c r="C4" s="33" t="s">
+      <c r="B4" s="35"/>
+      <c r="C4" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="35"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="33"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="33" t="s">
+      <c r="B5" s="35"/>
+      <c r="C5" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="35"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="33"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="32"/>
-      <c r="C6" s="33" t="s">
+      <c r="B6" s="35"/>
+      <c r="C6" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="35"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="33"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="31" t="s">
+      <c r="A7" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="32"/>
-      <c r="C7" s="33" t="s">
+      <c r="B7" s="35"/>
+      <c r="C7" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="34"/>
-      <c r="E7" s="34"/>
-      <c r="F7" s="35"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="33"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="31" t="s">
+      <c r="A8" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="32"/>
-      <c r="C8" s="33" t="s">
+      <c r="B8" s="35"/>
+      <c r="C8" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="35"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="33"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="31" t="s">
+      <c r="A9" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="32"/>
-      <c r="C9" s="33" t="s">
+      <c r="B9" s="35"/>
+      <c r="C9" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="34"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="35"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="33"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="31" t="s">
+      <c r="A10" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="32"/>
-      <c r="C10" s="33" t="s">
+      <c r="B10" s="35"/>
+      <c r="C10" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="35"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="33"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="36" t="s">
+      <c r="A12" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="32"/>
-      <c r="C12" s="32"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="32"/>
-      <c r="F12" s="32"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="35"/>
     </row>
     <row r="13" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="34"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="35"/>
+      <c r="B13" s="32"/>
+      <c r="C13" s="32"/>
+      <c r="D13" s="32"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="33"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="36" t="s">
+      <c r="A15" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="32"/>
-      <c r="C15" s="32"/>
-      <c r="D15" s="32"/>
-      <c r="E15" s="32"/>
-      <c r="F15" s="32"/>
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="35"/>
     </row>
     <row r="16" spans="1:6" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="31" t="s">
+      <c r="A16" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="32"/>
-      <c r="C16" s="33" t="s">
+      <c r="B16" s="35"/>
+      <c r="C16" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="35"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="33"/>
     </row>
     <row r="17" spans="1:6" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="31" t="s">
+      <c r="A17" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="32"/>
-      <c r="C17" s="33" t="s">
+      <c r="B17" s="35"/>
+      <c r="C17" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="35"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="33"/>
     </row>
     <row r="18" spans="1:6" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="31" t="s">
+      <c r="A18" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="32"/>
-      <c r="C18" s="33" t="s">
+      <c r="B18" s="35"/>
+      <c r="C18" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="35"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="33"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="36" t="s">
+      <c r="A20" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="32"/>
-      <c r="C20" s="32"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="32"/>
-      <c r="F20" s="32"/>
+      <c r="B20" s="35"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="35"/>
+      <c r="E20" s="35"/>
+      <c r="F20" s="35"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="38" t="s">
+      <c r="A21" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="40"/>
-      <c r="C21" s="38" t="s">
+      <c r="B21" s="37"/>
+      <c r="C21" s="36" t="s">
         <v>26</v>
       </c>
-      <c r="D21" s="40"/>
-      <c r="E21" s="38" t="s">
+      <c r="D21" s="37"/>
+      <c r="E21" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="F21" s="40"/>
+      <c r="F21" s="37"/>
     </row>
     <row r="22" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="33" t="s">
+      <c r="A22" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="B22" s="35"/>
-      <c r="C22" s="33" t="s">
+      <c r="B22" s="33"/>
+      <c r="C22" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="D22" s="35"/>
-      <c r="E22" s="33" t="s">
+      <c r="D22" s="33"/>
+      <c r="E22" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="F22" s="35"/>
+      <c r="F22" s="33"/>
     </row>
     <row r="23" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="33" t="s">
+      <c r="A23" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="B23" s="35"/>
-      <c r="C23" s="33" t="s">
+      <c r="B23" s="33"/>
+      <c r="C23" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D23" s="35"/>
-      <c r="E23" s="33" t="s">
+      <c r="D23" s="33"/>
+      <c r="E23" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="F23" s="35"/>
+      <c r="F23" s="33"/>
     </row>
     <row r="24" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="33" t="s">
+      <c r="A24" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="35"/>
-      <c r="C24" s="33" t="s">
+      <c r="B24" s="33"/>
+      <c r="C24" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="D24" s="35"/>
-      <c r="E24" s="33" t="s">
+      <c r="D24" s="33"/>
+      <c r="E24" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="F24" s="35"/>
+      <c r="F24" s="33"/>
     </row>
     <row r="25" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="33" t="s">
+      <c r="A25" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="35"/>
-      <c r="C25" s="33" t="s">
+      <c r="B25" s="33"/>
+      <c r="C25" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="D25" s="35"/>
-      <c r="E25" s="33" t="s">
+      <c r="D25" s="33"/>
+      <c r="E25" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="F25" s="35"/>
+      <c r="F25" s="33"/>
     </row>
     <row r="26" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="33" t="s">
+      <c r="A26" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="35"/>
-      <c r="C26" s="33" t="s">
+      <c r="B26" s="33"/>
+      <c r="C26" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="D26" s="35"/>
-      <c r="E26" s="33" t="s">
+      <c r="D26" s="33"/>
+      <c r="E26" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="F26" s="35"/>
+      <c r="F26" s="33"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="36" t="s">
+      <c r="A28" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="B28" s="32"/>
-      <c r="C28" s="32"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
+      <c r="B28" s="35"/>
+      <c r="C28" s="35"/>
+      <c r="D28" s="35"/>
+      <c r="E28" s="35"/>
+      <c r="F28" s="35"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="33" t="s">
+      <c r="A29" s="31" t="s">
         <v>684</v>
       </c>
-      <c r="B29" s="34"/>
-      <c r="C29" s="34"/>
-      <c r="D29" s="34"/>
-      <c r="E29" s="34"/>
-      <c r="F29" s="35"/>
+      <c r="B29" s="32"/>
+      <c r="C29" s="32"/>
+      <c r="D29" s="32"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="33"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="33" t="s">
+      <c r="A30" s="31" t="s">
         <v>42</v>
       </c>
-      <c r="B30" s="34"/>
-      <c r="C30" s="34"/>
-      <c r="D30" s="34"/>
-      <c r="E30" s="34"/>
-      <c r="F30" s="35"/>
+      <c r="B30" s="32"/>
+      <c r="C30" s="32"/>
+      <c r="D30" s="32"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="33"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="33" t="s">
+      <c r="A31" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="B31" s="34"/>
-      <c r="C31" s="34"/>
-      <c r="D31" s="34"/>
-      <c r="E31" s="34"/>
-      <c r="F31" s="35"/>
+      <c r="B31" s="32"/>
+      <c r="C31" s="32"/>
+      <c r="D31" s="32"/>
+      <c r="E31" s="32"/>
+      <c r="F31" s="33"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="33" t="s">
+      <c r="A32" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="B32" s="34"/>
-      <c r="C32" s="34"/>
-      <c r="D32" s="34"/>
-      <c r="E32" s="34"/>
-      <c r="F32" s="35"/>
+      <c r="B32" s="32"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="33"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="33" t="s">
+      <c r="A33" s="31" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="34"/>
-      <c r="C33" s="34"/>
-      <c r="D33" s="34"/>
-      <c r="E33" s="34"/>
-      <c r="F33" s="35"/>
+      <c r="B33" s="32"/>
+      <c r="C33" s="32"/>
+      <c r="D33" s="32"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="33"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="33" t="s">
+      <c r="A34" s="31" t="s">
         <v>46</v>
       </c>
-      <c r="B34" s="34"/>
-      <c r="C34" s="34"/>
-      <c r="D34" s="34"/>
-      <c r="E34" s="34"/>
-      <c r="F34" s="35"/>
+      <c r="B34" s="32"/>
+      <c r="C34" s="32"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="33"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="36" t="s">
+      <c r="A36" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="B36" s="32"/>
-      <c r="C36" s="32"/>
-      <c r="D36" s="32"/>
-      <c r="E36" s="32"/>
-      <c r="F36" s="32"/>
+      <c r="B36" s="35"/>
+      <c r="C36" s="35"/>
+      <c r="D36" s="35"/>
+      <c r="E36" s="35"/>
+      <c r="F36" s="35"/>
     </row>
     <row r="37" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="31" t="s">
+      <c r="A37" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="B37" s="32"/>
-      <c r="C37" s="33" t="s">
+      <c r="B37" s="35"/>
+      <c r="C37" s="31" t="s">
         <v>49</v>
       </c>
-      <c r="D37" s="34"/>
-      <c r="E37" s="34"/>
-      <c r="F37" s="35"/>
+      <c r="D37" s="32"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="33"/>
     </row>
     <row r="38" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="31" t="s">
+      <c r="A38" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="B38" s="32"/>
-      <c r="C38" s="33" t="s">
+      <c r="B38" s="35"/>
+      <c r="C38" s="31" t="s">
         <v>51</v>
       </c>
-      <c r="D38" s="34"/>
-      <c r="E38" s="34"/>
-      <c r="F38" s="35"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="33"/>
     </row>
     <row r="39" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="31" t="s">
+      <c r="A39" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="B39" s="32"/>
-      <c r="C39" s="33" t="s">
+      <c r="B39" s="35"/>
+      <c r="C39" s="31" t="s">
         <v>53</v>
       </c>
-      <c r="D39" s="34"/>
-      <c r="E39" s="34"/>
-      <c r="F39" s="35"/>
+      <c r="D39" s="32"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="33"/>
     </row>
     <row r="40" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="31" t="s">
+      <c r="A40" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="B40" s="32"/>
-      <c r="C40" s="33" t="s">
+      <c r="B40" s="35"/>
+      <c r="C40" s="31" t="s">
         <v>55</v>
       </c>
-      <c r="D40" s="34"/>
-      <c r="E40" s="34"/>
-      <c r="F40" s="35"/>
+      <c r="D40" s="32"/>
+      <c r="E40" s="32"/>
+      <c r="F40" s="33"/>
     </row>
     <row r="41" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="31" t="s">
+      <c r="A41" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="B41" s="32"/>
-      <c r="C41" s="33" t="s">
+      <c r="B41" s="35"/>
+      <c r="C41" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="D41" s="34"/>
-      <c r="E41" s="34"/>
-      <c r="F41" s="35"/>
+      <c r="D41" s="32"/>
+      <c r="E41" s="32"/>
+      <c r="F41" s="33"/>
     </row>
     <row r="42" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="31" t="s">
+      <c r="A42" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="B42" s="32"/>
-      <c r="C42" s="33" t="s">
+      <c r="B42" s="35"/>
+      <c r="C42" s="31" t="s">
         <v>59</v>
       </c>
-      <c r="D42" s="34"/>
-      <c r="E42" s="34"/>
-      <c r="F42" s="35"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="32"/>
+      <c r="F42" s="33"/>
     </row>
     <row r="43" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="31" t="s">
+      <c r="A43" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="B43" s="32"/>
-      <c r="C43" s="33" t="s">
+      <c r="B43" s="35"/>
+      <c r="C43" s="31" t="s">
         <v>61</v>
       </c>
-      <c r="D43" s="34"/>
-      <c r="E43" s="34"/>
-      <c r="F43" s="35"/>
+      <c r="D43" s="32"/>
+      <c r="E43" s="32"/>
+      <c r="F43" s="33"/>
     </row>
     <row r="44" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="31" t="s">
+      <c r="A44" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="B44" s="32"/>
-      <c r="C44" s="33" t="s">
+      <c r="B44" s="35"/>
+      <c r="C44" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="D44" s="34"/>
-      <c r="E44" s="34"/>
-      <c r="F44" s="35"/>
+      <c r="D44" s="32"/>
+      <c r="E44" s="32"/>
+      <c r="F44" s="33"/>
     </row>
     <row r="45" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="31" t="s">
+      <c r="A45" s="34" t="s">
         <v>64</v>
       </c>
-      <c r="B45" s="32"/>
-      <c r="C45" s="33" t="s">
+      <c r="B45" s="35"/>
+      <c r="C45" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="D45" s="34"/>
-      <c r="E45" s="34"/>
-      <c r="F45" s="35"/>
+      <c r="D45" s="32"/>
+      <c r="E45" s="32"/>
+      <c r="F45" s="33"/>
     </row>
     <row r="46" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="31" t="s">
+      <c r="A46" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="B46" s="32"/>
-      <c r="C46" s="33" t="s">
+      <c r="B46" s="35"/>
+      <c r="C46" s="31" t="s">
         <v>67</v>
       </c>
-      <c r="D46" s="34"/>
-      <c r="E46" s="34"/>
-      <c r="F46" s="35"/>
+      <c r="D46" s="32"/>
+      <c r="E46" s="32"/>
+      <c r="F46" s="33"/>
     </row>
     <row r="47" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="31" t="s">
+      <c r="A47" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="B47" s="32"/>
-      <c r="C47" s="33" t="s">
+      <c r="B47" s="35"/>
+      <c r="C47" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="D47" s="34"/>
-      <c r="E47" s="34"/>
-      <c r="F47" s="35"/>
+      <c r="D47" s="32"/>
+      <c r="E47" s="32"/>
+      <c r="F47" s="33"/>
     </row>
     <row r="48" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="31" t="s">
+      <c r="A48" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="B48" s="32"/>
-      <c r="C48" s="33" t="s">
+      <c r="B48" s="35"/>
+      <c r="C48" s="31" t="s">
         <v>71</v>
       </c>
-      <c r="D48" s="34"/>
-      <c r="E48" s="34"/>
-      <c r="F48" s="35"/>
+      <c r="D48" s="32"/>
+      <c r="E48" s="32"/>
+      <c r="F48" s="33"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="36" t="s">
+      <c r="A50" s="38" t="s">
         <v>72</v>
       </c>
-      <c r="B50" s="32"/>
-      <c r="C50" s="32"/>
-      <c r="D50" s="32"/>
-      <c r="E50" s="32"/>
-      <c r="F50" s="32"/>
+      <c r="B50" s="35"/>
+      <c r="C50" s="35"/>
+      <c r="D50" s="35"/>
+      <c r="E50" s="35"/>
+      <c r="F50" s="35"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
@@ -3450,11 +3450,11 @@
       <c r="B51" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C51" s="38" t="s">
+      <c r="C51" s="36" t="s">
         <v>26</v>
       </c>
-      <c r="D51" s="39"/>
-      <c r="E51" s="40"/>
+      <c r="D51" s="41"/>
+      <c r="E51" s="37"/>
       <c r="F51" s="2" t="s">
         <v>74</v>
       </c>
@@ -3466,11 +3466,11 @@
       <c r="B52" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C52" s="33" t="s">
+      <c r="C52" s="31" t="s">
         <v>77</v>
       </c>
-      <c r="D52" s="34"/>
-      <c r="E52" s="35"/>
+      <c r="D52" s="32"/>
+      <c r="E52" s="33"/>
       <c r="F52" s="1" t="s">
         <v>78</v>
       </c>
@@ -3482,11 +3482,11 @@
       <c r="B53" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C53" s="33" t="s">
+      <c r="C53" s="31" t="s">
         <v>81</v>
       </c>
-      <c r="D53" s="34"/>
-      <c r="E53" s="35"/>
+      <c r="D53" s="32"/>
+      <c r="E53" s="33"/>
       <c r="F53" s="1" t="s">
         <v>82</v>
       </c>
@@ -3498,11 +3498,11 @@
       <c r="B54" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C54" s="33" t="s">
+      <c r="C54" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="D54" s="34"/>
-      <c r="E54" s="35"/>
+      <c r="D54" s="32"/>
+      <c r="E54" s="33"/>
       <c r="F54" s="1" t="s">
         <v>86</v>
       </c>
@@ -3514,11 +3514,11 @@
       <c r="B55" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C55" s="33" t="s">
+      <c r="C55" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="D55" s="34"/>
-      <c r="E55" s="35"/>
+      <c r="D55" s="32"/>
+      <c r="E55" s="33"/>
       <c r="F55" s="1" t="s">
         <v>90</v>
       </c>
@@ -3530,11 +3530,11 @@
       <c r="B56" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C56" s="33" t="s">
+      <c r="C56" s="31" t="s">
         <v>685</v>
       </c>
-      <c r="D56" s="34"/>
-      <c r="E56" s="35"/>
+      <c r="D56" s="32"/>
+      <c r="E56" s="33"/>
       <c r="F56" s="1" t="s">
         <v>93</v>
       </c>
@@ -3546,17 +3546,85 @@
       <c r="B57" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C57" s="33" t="s">
+      <c r="C57" s="31" t="s">
         <v>96</v>
       </c>
-      <c r="D57" s="34"/>
-      <c r="E57" s="35"/>
+      <c r="D57" s="32"/>
+      <c r="E57" s="33"/>
       <c r="F57" s="1" t="s">
         <v>97</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="84">
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="C40:F40"/>
+    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C48:F48"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="C39:F39"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C8:F8"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C42:F42"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="C45:F45"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="C37:F37"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="C44:F44"/>
+    <mergeCell ref="C41:F41"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C46:F46"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C43:F43"/>
+    <mergeCell ref="E23:F23"/>
     <mergeCell ref="C57:E57"/>
     <mergeCell ref="C9:F9"/>
     <mergeCell ref="A43:B43"/>
@@ -3573,74 +3641,6 @@
     <mergeCell ref="C17:F17"/>
     <mergeCell ref="A44:B44"/>
     <mergeCell ref="C38:F38"/>
-    <mergeCell ref="C41:F41"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="C16:F16"/>
-    <mergeCell ref="A48:B48"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="A33:F33"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="C46:F46"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C43:F43"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="C45:F45"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="A36:F36"/>
-    <mergeCell ref="C7:F7"/>
-    <mergeCell ref="C37:F37"/>
-    <mergeCell ref="C18:F18"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="C44:F44"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="C39:F39"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C8:F8"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C42:F42"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="C56:E56"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="C40:F40"/>
-    <mergeCell ref="A15:F15"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C48:F48"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="C10:F10"/>
-    <mergeCell ref="A6:B6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3658,31 +3658,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="39" t="s">
         <v>98</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="40" t="s">
         <v>682</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="B4" s="32"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -3991,13 +3991,13 @@
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="36" t="s">
+      <c r="A24" s="38" t="s">
         <v>141</v>
       </c>
-      <c r="B24" s="32"/>
-      <c r="C24" s="32"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="32"/>
+      <c r="B24" s="35"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="35"/>
+      <c r="E24" s="35"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
@@ -4102,13 +4102,13 @@
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="36" t="s">
+      <c r="A32" s="38" t="s">
         <v>152</v>
       </c>
-      <c r="B32" s="32"/>
-      <c r="C32" s="32"/>
-      <c r="D32" s="32"/>
-      <c r="E32" s="32"/>
+      <c r="B32" s="35"/>
+      <c r="C32" s="35"/>
+      <c r="D32" s="35"/>
+      <c r="E32" s="35"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
@@ -4179,13 +4179,13 @@
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="36" t="s">
+      <c r="A38" s="38" t="s">
         <v>159</v>
       </c>
-      <c r="B38" s="32"/>
-      <c r="C38" s="32"/>
-      <c r="D38" s="32"/>
-      <c r="E38" s="32"/>
+      <c r="B38" s="35"/>
+      <c r="C38" s="35"/>
+      <c r="D38" s="35"/>
+      <c r="E38" s="35"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
@@ -4290,13 +4290,13 @@
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="36" t="s">
+      <c r="A46" s="38" t="s">
         <v>169</v>
       </c>
-      <c r="B46" s="32"/>
-      <c r="C46" s="32"/>
-      <c r="D46" s="32"/>
-      <c r="E46" s="32"/>
+      <c r="B46" s="35"/>
+      <c r="C46" s="35"/>
+      <c r="D46" s="35"/>
+      <c r="E46" s="35"/>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
@@ -4384,13 +4384,13 @@
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="36" t="s">
+      <c r="A53" s="38" t="s">
         <v>178</v>
       </c>
-      <c r="B53" s="32"/>
-      <c r="C53" s="32"/>
-      <c r="D53" s="32"/>
-      <c r="E53" s="32"/>
+      <c r="B53" s="35"/>
+      <c r="C53" s="35"/>
+      <c r="D53" s="35"/>
+      <c r="E53" s="35"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
@@ -4478,13 +4478,13 @@
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="36" t="s">
+      <c r="A60" s="38" t="s">
         <v>186</v>
       </c>
-      <c r="B60" s="32"/>
-      <c r="C60" s="32"/>
-      <c r="D60" s="32"/>
-      <c r="E60" s="32"/>
+      <c r="B60" s="35"/>
+      <c r="C60" s="35"/>
+      <c r="D60" s="35"/>
+      <c r="E60" s="35"/>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
@@ -4555,13 +4555,13 @@
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" s="36" t="s">
+      <c r="A66" s="38" t="s">
         <v>192</v>
       </c>
-      <c r="B66" s="32"/>
-      <c r="C66" s="32"/>
-      <c r="D66" s="32"/>
-      <c r="E66" s="32"/>
+      <c r="B66" s="35"/>
+      <c r="C66" s="35"/>
+      <c r="D66" s="35"/>
+      <c r="E66" s="35"/>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
@@ -4678,31 +4678,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="39" t="s">
         <v>201</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="40" t="s">
         <v>687</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="38" t="s">
         <v>202</v>
       </c>
-      <c r="B4" s="32"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -4790,13 +4790,13 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="36" t="s">
+      <c r="A11" s="38" t="s">
         <v>226</v>
       </c>
-      <c r="B11" s="32"/>
-      <c r="C11" s="32"/>
-      <c r="D11" s="32"/>
-      <c r="E11" s="32"/>
+      <c r="B11" s="35"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="35"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
@@ -4884,13 +4884,13 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="36" t="s">
+      <c r="A18" s="38" t="s">
         <v>247</v>
       </c>
-      <c r="B18" s="32"/>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
+      <c r="B18" s="35"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="35"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
@@ -4978,13 +4978,13 @@
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="36" t="s">
+      <c r="A25" s="38" t="s">
         <v>268</v>
       </c>
-      <c r="B25" s="32"/>
-      <c r="C25" s="32"/>
-      <c r="D25" s="32"/>
-      <c r="E25" s="32"/>
+      <c r="B25" s="35"/>
+      <c r="C25" s="35"/>
+      <c r="D25" s="35"/>
+      <c r="E25" s="35"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
@@ -5038,13 +5038,13 @@
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="36" t="s">
+      <c r="A30" s="38" t="s">
         <v>279</v>
       </c>
-      <c r="B30" s="32"/>
-      <c r="C30" s="32"/>
-      <c r="D30" s="32"/>
-      <c r="E30" s="32"/>
+      <c r="B30" s="35"/>
+      <c r="C30" s="35"/>
+      <c r="D30" s="35"/>
+      <c r="E30" s="35"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
@@ -5081,13 +5081,13 @@
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="36" t="s">
+      <c r="A34" s="38" t="s">
         <v>285</v>
       </c>
-      <c r="B34" s="32"/>
-      <c r="C34" s="32"/>
-      <c r="D34" s="32"/>
-      <c r="E34" s="32"/>
+      <c r="B34" s="35"/>
+      <c r="C34" s="35"/>
+      <c r="D34" s="35"/>
+      <c r="E34" s="35"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
@@ -5288,31 +5288,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="39" t="s">
         <v>322</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="40" t="s">
         <v>693</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="38" t="s">
         <v>323</v>
       </c>
-      <c r="B4" s="32"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
@@ -5731,37 +5731,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="39" t="s">
         <v>398</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="40" t="s">
         <v>399</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="38" t="s">
         <v>400</v>
       </c>
-      <c r="B4" s="32"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="35"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -5833,15 +5833,15 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="38" t="s">
         <v>418</v>
       </c>
-      <c r="B9" s="32"/>
-      <c r="C9" s="32"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
-      <c r="G9" s="32"/>
+      <c r="B9" s="35"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="35"/>
+      <c r="G9" s="35"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
@@ -5958,15 +5958,15 @@
       <c r="G15" s="1"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="36" t="s">
+      <c r="A17" s="38" t="s">
         <v>445</v>
       </c>
-      <c r="B17" s="32"/>
-      <c r="C17" s="32"/>
-      <c r="D17" s="32"/>
-      <c r="E17" s="32"/>
-      <c r="F17" s="32"/>
-      <c r="G17" s="32"/>
+      <c r="B17" s="35"/>
+      <c r="C17" s="35"/>
+      <c r="D17" s="35"/>
+      <c r="E17" s="35"/>
+      <c r="F17" s="35"/>
+      <c r="G17" s="35"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
@@ -6140,15 +6140,15 @@
       <c r="G26" s="1"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="36" t="s">
+      <c r="A28" s="38" t="s">
         <v>478</v>
       </c>
-      <c r="B28" s="32"/>
-      <c r="C28" s="32"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="32"/>
+      <c r="B28" s="35"/>
+      <c r="C28" s="35"/>
+      <c r="D28" s="35"/>
+      <c r="E28" s="35"/>
+      <c r="F28" s="35"/>
+      <c r="G28" s="35"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
@@ -6360,26 +6360,26 @@
       <c r="G39" s="1"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="36" t="s">
+      <c r="A41" s="38" t="s">
         <v>500</v>
       </c>
-      <c r="B41" s="32"/>
-      <c r="C41" s="32"/>
-      <c r="D41" s="32"/>
-      <c r="E41" s="32"/>
-      <c r="F41" s="32"/>
-      <c r="G41" s="32"/>
+      <c r="B41" s="35"/>
+      <c r="C41" s="35"/>
+      <c r="D41" s="35"/>
+      <c r="E41" s="35"/>
+      <c r="F41" s="35"/>
+      <c r="G41" s="35"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="43" t="s">
         <v>501</v>
       </c>
-      <c r="B42" s="32"/>
-      <c r="C42" s="32"/>
-      <c r="D42" s="32"/>
-      <c r="E42" s="32"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="32"/>
+      <c r="B42" s="35"/>
+      <c r="C42" s="35"/>
+      <c r="D42" s="35"/>
+      <c r="E42" s="35"/>
+      <c r="F42" s="35"/>
+      <c r="G42" s="35"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
@@ -6436,12 +6436,12 @@
       <c r="A47" s="42" t="s">
         <v>510</v>
       </c>
-      <c r="B47" s="32"/>
-      <c r="C47" s="32"/>
-      <c r="D47" s="32"/>
-      <c r="E47" s="32"/>
-      <c r="F47" s="32"/>
-      <c r="G47" s="32"/>
+      <c r="B47" s="35"/>
+      <c r="C47" s="35"/>
+      <c r="D47" s="35"/>
+      <c r="E47" s="35"/>
+      <c r="F47" s="35"/>
+      <c r="G47" s="35"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
@@ -6608,34 +6608,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="39" t="s">
         <v>532</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="44" t="s">
         <v>689</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="42" t="s">
         <v>533</v>
       </c>
-      <c r="B4" s="32"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -6721,11 +6721,11 @@
       <c r="A10" s="46" t="s">
         <v>557</v>
       </c>
-      <c r="B10" s="32"/>
-      <c r="C10" s="32"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32"/>
-      <c r="F10" s="32"/>
+      <c r="B10" s="35"/>
+      <c r="C10" s="35"/>
+      <c r="D10" s="35"/>
+      <c r="E10" s="35"/>
+      <c r="F10" s="35"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
@@ -6811,11 +6811,11 @@
       <c r="A16" s="49" t="s">
         <v>576</v>
       </c>
-      <c r="B16" s="32"/>
-      <c r="C16" s="32"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="32"/>
-      <c r="F16" s="32"/>
+      <c r="B16" s="35"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="35"/>
+      <c r="E16" s="35"/>
+      <c r="F16" s="35"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
@@ -6901,11 +6901,11 @@
       <c r="A22" s="48" t="s">
         <v>594</v>
       </c>
-      <c r="B22" s="32"/>
-      <c r="C22" s="32"/>
-      <c r="D22" s="32"/>
-      <c r="E22" s="32"/>
-      <c r="F22" s="32"/>
+      <c r="B22" s="35"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="35"/>
+      <c r="E22" s="35"/>
+      <c r="F22" s="35"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
@@ -6971,11 +6971,11 @@
       <c r="A27" s="47" t="s">
         <v>607</v>
       </c>
-      <c r="B27" s="32"/>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="32"/>
+      <c r="B27" s="35"/>
+      <c r="C27" s="35"/>
+      <c r="D27" s="35"/>
+      <c r="E27" s="35"/>
+      <c r="F27" s="35"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
@@ -7041,11 +7041,11 @@
       <c r="A32" s="45" t="s">
         <v>620</v>
       </c>
-      <c r="B32" s="32"/>
-      <c r="C32" s="32"/>
-      <c r="D32" s="32"/>
-      <c r="E32" s="32"/>
-      <c r="F32" s="32"/>
+      <c r="B32" s="35"/>
+      <c r="C32" s="35"/>
+      <c r="D32" s="35"/>
+      <c r="E32" s="35"/>
+      <c r="F32" s="35"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
@@ -7154,210 +7154,210 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="39" t="s">
         <v>639</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="44" t="s">
         <v>690</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="38" t="s">
         <v>640</v>
       </c>
-      <c r="B4" s="32"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
     </row>
     <row r="5" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="50" t="s">
         <v>641</v>
       </c>
-      <c r="B5" s="35"/>
-      <c r="C5" s="33" t="s">
+      <c r="B5" s="33"/>
+      <c r="C5" s="31" t="s">
         <v>642</v>
       </c>
-      <c r="D5" s="35"/>
+      <c r="D5" s="33"/>
     </row>
     <row r="6" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="50" t="s">
         <v>643</v>
       </c>
-      <c r="B6" s="35"/>
-      <c r="C6" s="33" t="s">
+      <c r="B6" s="33"/>
+      <c r="C6" s="31" t="s">
         <v>644</v>
       </c>
-      <c r="D6" s="35"/>
+      <c r="D6" s="33"/>
     </row>
     <row r="7" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="50" t="s">
         <v>645</v>
       </c>
-      <c r="B7" s="35"/>
-      <c r="C7" s="33" t="s">
+      <c r="B7" s="33"/>
+      <c r="C7" s="31" t="s">
         <v>646</v>
       </c>
-      <c r="D7" s="35"/>
+      <c r="D7" s="33"/>
     </row>
     <row r="8" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="50" t="s">
         <v>647</v>
       </c>
-      <c r="B8" s="35"/>
-      <c r="C8" s="33" t="s">
+      <c r="B8" s="33"/>
+      <c r="C8" s="31" t="s">
         <v>648</v>
       </c>
-      <c r="D8" s="35"/>
+      <c r="D8" s="33"/>
     </row>
     <row r="9" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="50" t="s">
         <v>649</v>
       </c>
-      <c r="B9" s="35"/>
-      <c r="C9" s="33" t="s">
+      <c r="B9" s="33"/>
+      <c r="C9" s="31" t="s">
         <v>650</v>
       </c>
-      <c r="D9" s="35"/>
+      <c r="D9" s="33"/>
     </row>
     <row r="10" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="50" t="s">
         <v>651</v>
       </c>
-      <c r="B10" s="35"/>
-      <c r="C10" s="33" t="s">
+      <c r="B10" s="33"/>
+      <c r="C10" s="31" t="s">
         <v>652</v>
       </c>
-      <c r="D10" s="35"/>
+      <c r="D10" s="33"/>
     </row>
     <row r="11" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="50" t="s">
         <v>653</v>
       </c>
-      <c r="B11" s="35"/>
-      <c r="C11" s="33" t="s">
+      <c r="B11" s="33"/>
+      <c r="C11" s="31" t="s">
         <v>654</v>
       </c>
-      <c r="D11" s="35"/>
+      <c r="D11" s="33"/>
     </row>
     <row r="12" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="50" t="s">
         <v>681</v>
       </c>
-      <c r="B12" s="35"/>
-      <c r="C12" s="33" t="s">
+      <c r="B12" s="33"/>
+      <c r="C12" s="31" t="s">
         <v>655</v>
       </c>
-      <c r="D12" s="35"/>
+      <c r="D12" s="33"/>
     </row>
     <row r="13" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="50" t="s">
         <v>656</v>
       </c>
-      <c r="B13" s="35"/>
-      <c r="C13" s="33" t="s">
+      <c r="B13" s="33"/>
+      <c r="C13" s="31" t="s">
         <v>657</v>
       </c>
-      <c r="D13" s="35"/>
+      <c r="D13" s="33"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="36" t="s">
+      <c r="A15" s="38" t="s">
         <v>658</v>
       </c>
-      <c r="B15" s="32"/>
-      <c r="C15" s="32"/>
-      <c r="D15" s="32"/>
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="35"/>
     </row>
     <row r="16" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="50" t="s">
         <v>659</v>
       </c>
-      <c r="B16" s="35"/>
-      <c r="C16" s="52" t="s">
+      <c r="B16" s="33"/>
+      <c r="C16" s="51" t="s">
         <v>660</v>
       </c>
-      <c r="D16" s="35"/>
+      <c r="D16" s="33"/>
     </row>
     <row r="17" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="50" t="s">
         <v>661</v>
       </c>
-      <c r="B17" s="35"/>
-      <c r="C17" s="51" t="s">
+      <c r="B17" s="33"/>
+      <c r="C17" s="52" t="s">
         <v>662</v>
       </c>
-      <c r="D17" s="35"/>
+      <c r="D17" s="33"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="36" t="s">
+      <c r="A19" s="38" t="s">
         <v>663</v>
       </c>
-      <c r="B19" s="32"/>
-      <c r="C19" s="32"/>
-      <c r="D19" s="32"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="35"/>
     </row>
     <row r="20" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="50" t="s">
         <v>664</v>
       </c>
-      <c r="B20" s="35"/>
-      <c r="C20" s="33" t="s">
+      <c r="B20" s="33"/>
+      <c r="C20" s="31" t="s">
         <v>665</v>
       </c>
-      <c r="D20" s="35"/>
+      <c r="D20" s="33"/>
     </row>
     <row r="21" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="50" t="s">
         <v>62</v>
       </c>
-      <c r="B21" s="35"/>
-      <c r="C21" s="33" t="s">
+      <c r="B21" s="33"/>
+      <c r="C21" s="31" t="s">
         <v>666</v>
       </c>
-      <c r="D21" s="35"/>
+      <c r="D21" s="33"/>
     </row>
     <row r="22" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="50" t="s">
         <v>507</v>
       </c>
-      <c r="B22" s="35"/>
-      <c r="C22" s="33" t="s">
+      <c r="B22" s="33"/>
+      <c r="C22" s="31" t="s">
         <v>667</v>
       </c>
-      <c r="D22" s="35"/>
+      <c r="D22" s="33"/>
     </row>
     <row r="23" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="50" t="s">
         <v>64</v>
       </c>
-      <c r="B23" s="35"/>
-      <c r="C23" s="33" t="s">
+      <c r="B23" s="33"/>
+      <c r="C23" s="31" t="s">
         <v>668</v>
       </c>
-      <c r="D23" s="35"/>
+      <c r="D23" s="33"/>
     </row>
     <row r="24" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="50" t="s">
         <v>669</v>
       </c>
-      <c r="B24" s="35"/>
-      <c r="C24" s="33" t="s">
+      <c r="B24" s="33"/>
+      <c r="C24" s="31" t="s">
         <v>670</v>
       </c>
-      <c r="D24" s="35"/>
+      <c r="D24" s="33"/>
     </row>
     <row r="25" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="50"/>
-      <c r="B25" s="35"/>
-      <c r="C25" s="33"/>
-      <c r="D25" s="35"/>
+      <c r="B25" s="33"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="33"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="21"/>
@@ -7367,6 +7367,29 @@
     </row>
   </sheetData>
   <mergeCells count="39">
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="A19:D19"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A22:B22"/>
@@ -7383,29 +7406,6 @@
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="C16:D16"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C20:D20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>